<commit_message>
ENgineering analysis for structure, floatation, and stability
</commit_message>
<xml_diff>
--- a/rev7_AluminumHull_Fusion/BOM_rev7.xlsx
+++ b/rev7_AluminumHull_Fusion/BOM_rev7.xlsx
@@ -622,7 +622,7 @@
     <row r="1" ht="17.35" customHeight="1" s="31">
       <c r="A1" s="32" t="inlineStr">
         <is>
-          <t>DIY Mini-Airboat — BOM summary, rev 7 (riveted aluminum hull)</t>
+          <t>Straddle Dart — BOM summary, rev 7 (riveted aluminum hull)</t>
         </is>
       </c>
     </row>
@@ -714,19 +714,19 @@
         </is>
       </c>
       <c r="B7" s="36">
-        <f>'Everything else'!F93</f>
+        <f>'Everything else'!F102</f>
         <v/>
       </c>
       <c r="C7" s="37">
-        <f>'Everything else'!G93</f>
+        <f>'Everything else'!G102</f>
         <v/>
       </c>
       <c r="D7" s="37">
-        <f>'Everything else'!G94</f>
+        <f>'Everything else'!G103</f>
         <v/>
       </c>
       <c r="E7" s="37">
-        <f>'Everything else'!G95</f>
+        <f>'Everything else'!G104</f>
         <v/>
       </c>
     </row>
@@ -830,7 +830,7 @@
         </is>
       </c>
       <c r="B15" s="46" t="n">
-        <v>1159</v>
+        <v>1160</v>
       </c>
       <c r="C15" s="33" t="inlineStr">
         <is>
@@ -926,7 +926,7 @@
     <row r="1" ht="17.35" customHeight="1" s="31">
       <c r="A1" s="32" t="inlineStr">
         <is>
-          <t>DIY Mini-Airboat — Hull BOM (riveted aluminum) (rev 7)</t>
+          <t>Straddle Dart — Hull BOM (riveted aluminum) (rev 7)</t>
         </is>
       </c>
     </row>
@@ -993,7 +993,7 @@
     <row r="5" ht="23.85" customHeight="1" s="31">
       <c r="A5" s="50" t="inlineStr">
         <is>
-          <t>5052-H32 aluminum sheet 0.090 in, 60 x 144 in</t>
+          <t>5052-H32 aluminum sheet 0.125 in, 60 x 144 in</t>
         </is>
       </c>
       <c r="B5" s="50" t="inlineStr">
@@ -1010,14 +1010,14 @@
         </is>
       </c>
       <c r="E5" s="53" t="n">
-        <v>450</v>
+        <v>625</v>
       </c>
       <c r="F5" s="54">
         <f>C5*E5</f>
         <v/>
       </c>
       <c r="G5" s="55" t="n">
-        <v>97.59999999999999</v>
+        <v>135.6</v>
       </c>
       <c r="H5" s="52" t="inlineStr">
         <is>
@@ -1027,7 +1027,7 @@
       <c r="I5" s="52" t="n"/>
       <c r="J5" s="50" t="inlineStr">
         <is>
-          <t>Centerline seam over the center stringer; transverse butt seam with doubler at frame 120</t>
+          <t>Was 0.090: ISO 12215-5 check (Structural Checks 8c). Centerline seam over the center stringer; transverse butt seam with doubler at frame 120</t>
         </is>
       </c>
     </row>
@@ -1154,11 +1154,11 @@
       </c>
       <c r="B9" s="50" t="inlineStr">
         <is>
-          <t>7 frames + transom frame</t>
+          <t>10 frames (x 12, 24, 36, 48, 60, 72, 84, 96, 111.5, 120 in) + transom frame</t>
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D9" s="52" t="inlineStr">
         <is>
@@ -1173,7 +1173,7 @@
         <v/>
       </c>
       <c r="G9" s="55" t="n">
-        <v>24.8</v>
+        <v>38.9</v>
       </c>
       <c r="H9" s="52" t="inlineStr">
         <is>
@@ -1183,7 +1183,7 @@
       <c r="I9" s="52" t="n"/>
       <c r="J9" s="50" t="inlineStr">
         <is>
-          <t>1 x 3/4 in limber notch at the skin in every bay of every frame; deburr and prime the cut edges</t>
+          <t>Frames at 60, 84 and 111.5 in added for the 0.125 bottom (ISO 12215-5). 1 x 3/4 in limber notch at the skin in every bay of every frame; deburr and prime the cut edges</t>
         </is>
       </c>
     </row>
@@ -1379,7 +1379,7 @@
     <row r="15" ht="23.85" customHeight="1" s="31">
       <c r="A15" s="50" t="inlineStr">
         <is>
-          <t>6061 angle 1-1/2 x 1-1/2 x 1/8 in (2) + 5052 sheet 1/8 in for nose cap</t>
+          <t>5052-H32 sheet 1/8 in: two chine guards brake-formed to 135 deg (12.5 ft) + bent nose cap</t>
         </is>
       </c>
       <c r="B15" s="50" t="inlineStr">
@@ -1396,7 +1396,7 @@
         </is>
       </c>
       <c r="E15" s="53" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
       <c r="F15" s="54">
         <f>C15*E15</f>
@@ -1411,7 +1411,11 @@
         </is>
       </c>
       <c r="I15" s="52" t="n"/>
-      <c r="J15" s="50" t="n"/>
+      <c r="J15" s="50" t="inlineStr">
+        <is>
+          <t>Guards brake-formed at the shop with the chine bends (were 6061 angles opened to 135 deg by hand)</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="31">
       <c r="A16" s="50" t="inlineStr">
@@ -1466,7 +1470,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>2500</v>
+        <v>2400</v>
       </c>
       <c r="D17" s="52" t="inlineStr">
         <is>
@@ -1481,7 +1485,7 @@
         <v/>
       </c>
       <c r="G17" s="55" t="n">
-        <v>5</v>
+        <v>4.8</v>
       </c>
       <c r="H17" s="52" t="inlineStr">
         <is>
@@ -1491,7 +1495,7 @@
       <c r="I17" s="52" t="n"/>
       <c r="J17" s="50" t="inlineStr">
         <is>
-          <t>Never open-end or steel-mandrel rivets</t>
+          <t>Double rows: 3/4 in pitch on the bottom seams and chine laps, 1 in on laps above the waterline. Never open-end or steel-mandrel rivets</t>
         </is>
       </c>
     </row>
@@ -1613,12 +1617,12 @@
     <row r="21" ht="15" customHeight="1" s="31">
       <c r="A21" s="50" t="inlineStr">
         <is>
-          <t>Self-etching primer + marine topcoat (olive drab)</t>
+          <t>Self-etching primer</t>
         </is>
       </c>
       <c r="B21" s="50" t="inlineStr">
         <is>
-          <t>Inside and out</t>
+          <t>Faying surfaces and cut edges only; the hull stays bare 5052 (topcoat optional later)</t>
         </is>
       </c>
       <c r="C21" s="51" t="n">
@@ -1630,14 +1634,14 @@
         </is>
       </c>
       <c r="E21" s="53" t="n">
-        <v>260</v>
+        <v>60</v>
       </c>
       <c r="F21" s="54">
         <f>C21*E21</f>
         <v/>
       </c>
       <c r="G21" s="55" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H21" s="52" t="inlineStr">
         <is>
@@ -1793,7 +1797,7 @@
     <row r="1" ht="17.35" customHeight="1" s="31">
       <c r="A1" s="32" t="inlineStr">
         <is>
-          <t>DIY Mini-Airboat — Drivetrain BOM (rev 7)</t>
+          <t>Straddle Dart — Drivetrain BOM (rev 7)</t>
         </is>
       </c>
     </row>
@@ -1860,12 +1864,12 @@
     <row r="5" ht="23.85" customHeight="1" s="31">
       <c r="A5" s="50" t="inlineStr">
         <is>
-          <t>Suzuki G13 1.3 L engine (junkyard), dressed</t>
+          <t>Suzuki G13B 1.3 L DOHC 16-valve engine, dressed</t>
         </is>
       </c>
       <c r="B5" s="50" t="inlineStr">
         <is>
-          <t>1995-2001 Geo/Chevy Metro 1.3 or Suzuki Swift; with flywheel, starter, alternator, intake, ECU/harness</t>
+          <t>1989-94 Suzuki Swift GT/GTi (US) or a JDM Cultus GT-i import; with flywheel, starter, alternator, intake, ECU and harness</t>
         </is>
       </c>
       <c r="C5" s="51" t="n">
@@ -1877,14 +1881,14 @@
         </is>
       </c>
       <c r="E5" s="53" t="n">
-        <v>600</v>
+        <v>1200</v>
       </c>
       <c r="F5" s="54">
         <f>C5*E5</f>
         <v/>
       </c>
       <c r="G5" s="55" t="n">
-        <v>179</v>
+        <v>194</v>
       </c>
       <c r="H5" s="52" t="inlineStr">
         <is>
@@ -1898,7 +1902,7 @@
       </c>
       <c r="J5" s="50" t="inlineStr">
         <is>
-          <t>Weight is the CAD placeholder: verify on a scale</t>
+          <t>About 100 hp at 6,500 rpm, about 83 lb-ft. Weight is the CAD placeholder + 15 lb for the twin-cam head: verify weight and head clearances on the engine bought</t>
         </is>
       </c>
     </row>
@@ -1984,7 +1988,7 @@
       </c>
       <c r="B8" s="50" t="inlineStr">
         <is>
-          <t>3/8 in 6061 plate + shroud, machined to the G13 pattern, starter boss</t>
+          <t>3/8 in 6061 plate + shroud, machined to the G13-family pattern (G13B), starter boss</t>
         </is>
       </c>
       <c r="C8" s="51" t="n">
@@ -2202,7 +2206,7 @@
       <c r="I13" s="52" t="n"/>
       <c r="J13" s="50" t="inlineStr">
         <is>
-          <t>Confirm width with Gates design data for 74 lb-ft</t>
+          <t>Confirm width with Gates design data for the G13B (83 lb-ft, 6,500 rpm); may need a wider HTD belt or Poly Chain GT Carbon</t>
         </is>
       </c>
     </row>
@@ -2250,7 +2254,7 @@
     <row r="15" ht="15" customHeight="1" s="31">
       <c r="A15" s="50" t="inlineStr">
         <is>
-          <t>Prop shaft 1-1/2 in 4140, 20 in, keyed</t>
+          <t>Prop shaft 1-1/2 in 4140 pre-hardened (28-32 HRC), 20 in, keyed</t>
         </is>
       </c>
       <c r="B15" s="50" t="inlineStr">
@@ -2267,7 +2271,7 @@
         </is>
       </c>
       <c r="E15" s="53" t="n">
-        <v>110</v>
+        <v>140</v>
       </c>
       <c r="F15" s="54">
         <f>C15*E15</f>
@@ -2282,7 +2286,11 @@
         </is>
       </c>
       <c r="I15" s="52" t="n"/>
-      <c r="J15" s="50" t="n"/>
+      <c r="J15" s="50" t="inlineStr">
+        <is>
+          <t>Pre-hardened for gyroscopic bending in hard turns; carry thrust on a shoulder or clamped collar, not set screws alone</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="31">
       <c r="A16" s="50" t="inlineStr">
@@ -2440,11 +2448,11 @@
       </c>
       <c r="B20" s="50" t="inlineStr">
         <is>
-          <t>A-frame legs and crossbars</t>
+          <t>A-frame legs and aft crossbar</t>
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="D20" s="52" t="inlineStr">
         <is>
@@ -2459,7 +2467,7 @@
         <v/>
       </c>
       <c r="G20" s="55" t="n">
-        <v>17.8</v>
+        <v>16.1</v>
       </c>
       <c r="H20" s="52" t="inlineStr">
         <is>
@@ -2658,7 +2666,7 @@
       </c>
       <c r="J25" s="50" t="inlineStr">
         <is>
-          <t>Price from Warp Drive page; confirm rotation, hub pattern and weight before ordering</t>
+          <t>Price from Warp Drive page; confirm rotation, hub pattern and weight before ordering. G13B: pitch for 6,000-6,300 rpm at full throttle standing still</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2746,11 @@
         </is>
       </c>
       <c r="I27" s="52" t="n"/>
-      <c r="J27" s="50" t="n"/>
+      <c r="J27" s="50" t="inlineStr">
+        <is>
+          <t>Civic radiator suits engines of about 100 hp; watch coolant temperature on a long static run</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="31">
       <c r="A28" s="50" t="inlineStr">
@@ -3019,7 +3031,7 @@
       <c r="I35" s="52" t="n"/>
       <c r="J35" s="50" t="inlineStr">
         <is>
-          <t>Measure the G13 mount bosses first</t>
+          <t>Measure the G13B mount bosses before drilling the engine-side brackets</t>
         </is>
       </c>
     </row>
@@ -3240,7 +3252,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J96"/>
+  <dimension ref="A1:J105"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="46" customWidth="1" style="30" min="1" max="1"/>
@@ -3256,7 +3268,7 @@
     <row r="1" ht="17.35" customHeight="1" s="31">
       <c r="A1" s="32" t="inlineStr">
         <is>
-          <t>DIY Mini-Airboat — Everything else BOM: cage, rudders, steering, seating, controls, flotation, electrical, safety (rev 7)</t>
+          <t>Straddle Dart — Everything else BOM: cage, rudders, steering, seating, controls, flotation, electrical, safety (rev 7)</t>
         </is>
       </c>
     </row>
@@ -3339,7 +3351,7 @@
     <row r="6" ht="15" customHeight="1" s="31">
       <c r="A6" s="50" t="inlineStr">
         <is>
-          <t>Steel tube 1 in x 0.049 in</t>
+          <t>Steel DOM tube 1 in x 0.083 in (yield 50 ksi or better)</t>
         </is>
       </c>
       <c r="B6" s="50" t="inlineStr">
@@ -3356,14 +3368,14 @@
         </is>
       </c>
       <c r="E6" s="56" t="n">
-        <v>3.5</v>
+        <v>6</v>
       </c>
       <c r="F6" s="54">
         <f>C6*E6</f>
         <v/>
       </c>
       <c r="G6" s="55" t="n">
-        <v>18.8</v>
+        <v>30.9</v>
       </c>
       <c r="H6" s="52" t="inlineStr">
         <is>
@@ -3371,7 +3383,11 @@
         </is>
       </c>
       <c r="I6" s="52" t="n"/>
-      <c r="J6" s="50" t="n"/>
+      <c r="J6" s="50" t="inlineStr">
+        <is>
+          <t>Was 1 x .049: the hoops carry rudder, steering and screen loads in bending (Structural Checks)</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="31">
       <c r="A7" s="50" t="inlineStr">
@@ -3381,7 +3397,7 @@
       </c>
       <c r="B7" s="50" t="inlineStr">
         <is>
-          <t>Roll two 72.4 in hoops</t>
+          <t>Roll two 72.4 in DOM hoops</t>
         </is>
       </c>
       <c r="C7" s="51" t="n">
@@ -3417,16 +3433,16 @@
     <row r="8" ht="15" customHeight="1" s="31">
       <c r="A8" s="50" t="inlineStr">
         <is>
-          <t>Steel tube 1 in x 0.065 in</t>
+          <t>Steel DOM tube 1 in x 0.065 in (yield 50 ksi or better)</t>
         </is>
       </c>
       <c r="B8" s="50" t="inlineStr">
         <is>
-          <t>Cage legs, base rails, rudder rails</t>
+          <t>Cage legs, base rails, rudder rails, 8 longitudinals, aft screen bars, 2 side-bay diagonals</t>
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="D8" s="52" t="inlineStr">
         <is>
@@ -3434,14 +3450,14 @@
         </is>
       </c>
       <c r="E8" s="56" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F8" s="54">
         <f>C8*E8</f>
         <v/>
       </c>
       <c r="G8" s="55" t="n">
-        <v>15.5</v>
+        <v>29.8</v>
       </c>
       <c r="H8" s="52" t="inlineStr">
         <is>
@@ -3449,21 +3465,25 @@
         </is>
       </c>
       <c r="I8" s="52" t="n"/>
-      <c r="J8" s="50" t="n"/>
+      <c r="J8" s="50" t="inlineStr">
+        <is>
+          <t>Longitudinals and aft bars were EMT; diagonals added (Structural Checks)</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="31">
       <c r="A9" s="50" t="inlineStr">
         <is>
-          <t>EMT conduit 3/4 in and 1/2 in, 10 ft sticks</t>
+          <t>EMT conduit 1/2 in, 10 ft sticks</t>
         </is>
       </c>
       <c r="B9" s="50" t="inlineStr">
         <is>
-          <t>Longitudinals (8) and face bars (4)</t>
+          <t>Front screen bars (2)</t>
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D9" s="52" t="inlineStr">
         <is>
@@ -3478,7 +3498,7 @@
         <v/>
       </c>
       <c r="G9" s="55" t="n">
-        <v>10.3</v>
+        <v>3.3</v>
       </c>
       <c r="H9" s="52" t="inlineStr">
         <is>
@@ -3741,12 +3761,12 @@
     <row r="17" ht="15" customHeight="1" s="31">
       <c r="A17" s="50" t="inlineStr">
         <is>
-          <t>Tie bar, pushrod, 4 rod ends, lever pivot</t>
+          <t>Steering linkage: 2 aft horns, tie bar and drive link (5/8 x .065 steel, 4 rod ends), bellcrank (1/4 steel, 3.5 / 4 in arms) on a 3/8 x 1.5 steel bracket welded to the aft hoop, 1 x .065 DOM long rod (8.5 ft) with 2 rod ends, 3/8 SS pins</t>
         </is>
       </c>
       <c r="B17" s="50" t="inlineStr">
         <is>
-          <t>Horns to the left-hand steering lever</t>
+          <t>Rudders to the left-hand steering lever; every link straight and pinned at both ends</t>
         </is>
       </c>
       <c r="C17" s="51" t="n">
@@ -3758,14 +3778,14 @@
         </is>
       </c>
       <c r="E17" s="53" t="n">
-        <v>130</v>
+        <v>190</v>
       </c>
       <c r="F17" s="54">
         <f>C17*E17</f>
         <v/>
       </c>
       <c r="G17" s="55" t="n">
-        <v>4.6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H17" s="52" t="inlineStr">
         <is>
@@ -3773,7 +3793,11 @@
         </is>
       </c>
       <c r="I17" s="52" t="n"/>
-      <c r="J17" s="50" t="n"/>
+      <c r="J17" s="50" t="inlineStr">
+        <is>
+          <t>Replaces the dog-legged pushrod, which would have bent (Structural Checks, finding 1); notch the aft screen mesh round the bracket</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="31">
       <c r="A18" s="57" t="inlineStr">
@@ -4061,12 +4085,12 @@
     <row r="26" ht="15" customHeight="1" s="31">
       <c r="A26" s="50" t="inlineStr">
         <is>
-          <t>Footrest ladder</t>
+          <t>Footrest, two foot ladders (6061 solid 1 in rod, welded)</t>
         </is>
       </c>
       <c r="B26" s="50" t="inlineStr">
         <is>
-          <t>5 rungs, x = 104.5-123 in</t>
+          <t>Left rails 7.5 and 12.5 in to port, right rails 7.5 and 14.5 in to starboard; 5 rungs each at x 105.5-117.5 in, rising 22.7 deg to the bow shelf; 8 foot plates 3/16</t>
         </is>
       </c>
       <c r="C26" s="51" t="n">
@@ -4078,14 +4102,14 @@
         </is>
       </c>
       <c r="E26" s="53" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="F26" s="54">
         <f>C26*E26</f>
         <v/>
       </c>
       <c r="G26" s="55" t="n">
-        <v>4</v>
+        <v>6.5</v>
       </c>
       <c r="H26" s="52" t="inlineStr">
         <is>
@@ -4093,7 +4117,11 @@
         </is>
       </c>
       <c r="I26" s="52" t="n"/>
-      <c r="J26" s="50" t="n"/>
+      <c r="J26" s="50" t="inlineStr">
+        <is>
+          <t>A landing for each foot like motorcycle pegs; the throttle pedal clamps to any right-ladder rung</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="31">
       <c r="A27" s="50" t="inlineStr">
@@ -4103,7 +4131,7 @@
       </c>
       <c r="B27" s="50" t="inlineStr">
         <is>
-          <t>Clamps to any ladder rung; cable arm, torsion return spring, rest stop</t>
+          <t>Clamps to any rung of the right foot ladder (centred 10.75 in to starboard); cable arm, torsion return spring, rest stop</t>
         </is>
       </c>
       <c r="C27" s="51" t="n">
@@ -4144,7 +4172,7 @@
       </c>
       <c r="B28" s="50" t="inlineStr">
         <is>
-          <t>Port side, left hand</t>
+          <t>Port side, left hand; 1.5 in outboard of the original position (clear of the left knee)</t>
         </is>
       </c>
       <c r="C28" s="51" t="n">
@@ -5181,7 +5209,7 @@
     <row r="57" ht="35.05" customHeight="1" s="31">
       <c r="A57" s="50" t="inlineStr">
         <is>
-          <t>Bench clips (4), battery tray + strap, steering pivot base + bushings, ladder foot plates (4), engine-guard angle + stays</t>
+          <t>Bench clips (4), battery tray + strap, steering pivot base + bushings, engine-guard angle + stays (ladder foot plates: see the footrest line)</t>
         </is>
       </c>
       <c r="B57" s="50" t="n"/>
@@ -5300,7 +5328,7 @@
       </c>
       <c r="B61" s="50" t="inlineStr">
         <is>
-          <t>2 x 2 x 1/8 sq tube posts, top rail and cross arms (14 ft); 2 x 3 x 1/8 inner rail (3 ft); 1-1/4 x .120 round tube knee braces and diagonal (8 ft); 3/8 clips; 1/4 base and backing plates</t>
+          <t>2 x 2 x 3/16 sq tube posts, top rail and cross arms (14 ft); 2 x 3 x 3/16 inner rail (3 ft); 1-1/2 x .188 round tube knee braces (rolled to about 19 in radius) and diagonal (8 ft); 3/8 clips; 1/4 base and backing plates</t>
         </is>
       </c>
       <c r="C61" s="51" t="n">
@@ -5312,14 +5340,14 @@
         </is>
       </c>
       <c r="E61" s="53" t="n">
-        <v>260</v>
+        <v>340</v>
       </c>
       <c r="F61" s="54">
         <f>C61*E61</f>
         <v/>
       </c>
       <c r="G61" s="55" t="n">
-        <v>16.2</v>
+        <v>23.1</v>
       </c>
       <c r="H61" s="52" t="inlineStr">
         <is>
@@ -5329,19 +5357,19 @@
       <c r="I61" s="52" t="n"/>
       <c r="J61" s="50" t="inlineStr">
         <is>
-          <t>Bolts to frame x96 and backing plates on the hull side; 11 in leg space</t>
+          <t>Bolts to frame x96 and backing plates on the hull side; braces bowed 2.5 in outboard for a large leg; 3/16 walls for the 600 lb hand-hold (Structural Checks)</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="31">
       <c r="A62" s="50" t="inlineStr">
         <is>
-          <t>Armrest pad</t>
+          <t>Console top, skins and dash hood, 5052</t>
         </is>
       </c>
       <c r="B62" s="50" t="inlineStr">
         <is>
-          <t>1/2 in ply base, 2 in foam, marine vinyl</t>
+          <t>1/8 in top (13 x 21 in); 0.063 in front and outboard skins; 0.063 in hood (visor, cheeks, arched top) folded and riveted; grommets for the dash loom and bow loom</t>
         </is>
       </c>
       <c r="C62" s="51" t="n">
@@ -5349,18 +5377,18 @@
       </c>
       <c r="D62" s="52" t="inlineStr">
         <is>
-          <t>ea</t>
+          <t>lot</t>
         </is>
       </c>
       <c r="E62" s="53" t="n">
-        <v>35</v>
+        <v>180</v>
       </c>
       <c r="F62" s="54">
         <f>C62*E62</f>
         <v/>
       </c>
       <c r="G62" s="55" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H62" s="52" t="inlineStr">
         <is>
@@ -5370,19 +5398,19 @@
       <c r="I62" s="52" t="n"/>
       <c r="J62" s="50" t="inlineStr">
         <is>
-          <t>Height set by drv_armrest_h</t>
+          <t>Hood and top screwed with tamper-proof Torx; gauge and switch backs sealed inside</t>
         </is>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="31">
       <c r="A63" s="50" t="inlineStr">
         <is>
-          <t>Grip (hand-hold), Hurst style</t>
+          <t>Console fiddle rail, 6061 flat bar 1/8 x 1-1/2</t>
         </is>
       </c>
       <c r="B63" s="50" t="inlineStr">
         <is>
-          <t>1 in 316 SS rod, bent, welded into the inner rail; 1-7/8 in white ball knob</t>
+          <t>Raised 1/2 in edge on the aft, inboard and forward edges of the console top (about 29 in); riveted to the cross arms and inner rail; top edges rounded</t>
         </is>
       </c>
       <c r="C63" s="51" t="n">
@@ -5390,18 +5418,18 @@
       </c>
       <c r="D63" s="52" t="inlineStr">
         <is>
-          <t>ea</t>
+          <t>lot</t>
         </is>
       </c>
       <c r="E63" s="53" t="n">
-        <v>55</v>
+        <v>15</v>
       </c>
       <c r="F63" s="54">
         <f>C63*E63</f>
         <v/>
       </c>
       <c r="G63" s="55" t="n">
-        <v>1.2</v>
+        <v>0.5</v>
       </c>
       <c r="H63" s="52" t="inlineStr">
         <is>
@@ -5411,38 +5439,38 @@
       <c r="I63" s="52" t="n"/>
       <c r="J63" s="50" t="inlineStr">
         <is>
-          <t>Sized for about 600 lbf; knob position from drv_reach</t>
+          <t>Keeps small things from rolling or sliding off, like a galley table</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="31">
       <c r="A64" s="50" t="inlineStr">
         <is>
-          <t>Dash panel and stalk</t>
+          <t>Knee brace pads</t>
         </is>
       </c>
       <c r="B64" s="50" t="inlineStr">
         <is>
-          <t>1/8 in 6061 panel, 1 in tube stalk; tilted 56 deg, turned 33 deg</t>
+          <t>1 in closed-cell foam (minicell) on both braces, UV-treated PU-coated 1000D Cordura or marine vinyl cover, Velcro or laced seam</t>
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D64" s="52" t="inlineStr">
         <is>
-          <t>lot</t>
+          <t>ea</t>
         </is>
       </c>
       <c r="E64" s="53" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="F64" s="54">
         <f>C64*E64</f>
         <v/>
       </c>
       <c r="G64" s="55" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="H64" s="52" t="inlineStr">
         <is>
@@ -5452,19 +5480,19 @@
       <c r="I64" s="52" t="n"/>
       <c r="J64" s="50" t="inlineStr">
         <is>
-          <t>Not a hand-hold</t>
+          <t>Replaceable covers; plain nylon Cordura fades in Florida sun</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="50" t="inlineStr">
         <is>
-          <t>12 V socket and USB-A 5 V / 3 A charger, marine</t>
+          <t>Life-jacket hook, 316 stainless</t>
         </is>
       </c>
       <c r="B65" s="50" t="inlineStr">
         <is>
-          <t>With hinged rubber flaps</t>
+          <t>J-hook riveted inside the outboard skin, 22 in up, 2.4 in reach</t>
         </is>
       </c>
       <c r="C65" s="51" t="n">
@@ -5472,18 +5500,18 @@
       </c>
       <c r="D65" s="52" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>ea</t>
         </is>
       </c>
       <c r="E65" s="53" t="n">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="F65" s="54">
         <f>C65*E65</f>
         <v/>
       </c>
       <c r="G65" s="55" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="H65" s="52" t="inlineStr">
         <is>
@@ -5493,23 +5521,23 @@
       <c r="I65" s="52" t="n"/>
       <c r="J65" s="50" t="inlineStr">
         <is>
-          <t>Both on the hub 20 A outlet circuit</t>
+          <t>Keeps a PFD in the sheltered cabinet, clear of the side diagonal</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="50" t="inlineStr">
         <is>
-          <t>Phone holder, swivel</t>
+          <t>Swamped-boat warning labels</t>
         </is>
       </c>
       <c r="B66" s="50" t="inlineStr">
         <is>
-          <t>Portrait or landscape (drv_phone_rot)</t>
+          <t>6 x 4 in UV-laminated marine vinyl, printed from Labels/Swamped_Warning_Label.svg</t>
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D66" s="52" t="inlineStr">
         <is>
@@ -5517,32 +5545,36 @@
         </is>
       </c>
       <c r="E66" s="53" t="n">
-        <v>35</v>
+        <v>8</v>
       </c>
       <c r="F66" s="54">
         <f>C66*E66</f>
         <v/>
       </c>
       <c r="G66" s="55" t="n">
-        <v>0.6</v>
+        <v>0.05</v>
       </c>
       <c r="H66" s="52" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="I66" s="52" t="n"/>
-      <c r="J66" s="50" t="n"/>
+      <c r="J66" s="50" t="inlineStr">
+        <is>
+          <t>Helm (console top, by the capacity label) and inside each side of the bench; stability report Finding 1</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="50" t="inlineStr">
         <is>
-          <t>Light switch panel</t>
+          <t>Cup holder, drop-in, drained</t>
         </is>
       </c>
       <c r="B67" s="50" t="inlineStr">
         <is>
-          <t>2 sealed OFF-LO-MED-HI rotary switches (light bar, searchlight) + nav-light rocker, DT12 connector</t>
+          <t>Stainless or nylon, 3.4 in bore, 2.75 in deep (shallow over the thigh)</t>
         </is>
       </c>
       <c r="C67" s="51" t="n">
@@ -5554,14 +5586,14 @@
         </is>
       </c>
       <c r="E67" s="53" t="n">
-        <v>85</v>
+        <v>20</v>
       </c>
       <c r="F67" s="54">
         <f>C67*E67</f>
         <v/>
       </c>
       <c r="G67" s="55" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="H67" s="52" t="inlineStr">
         <is>
@@ -5571,38 +5603,38 @@
       <c r="I67" s="52" t="n"/>
       <c r="J67" s="50" t="inlineStr">
         <is>
-          <t>On the aft cross arm; the rotaries set the dimmers in the battery bay</t>
+          <t>Just forward of the grip</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="50" t="inlineStr">
         <is>
-          <t>Bubble inclinometers</t>
+          <t>Armrest, hinged</t>
         </is>
       </c>
       <c r="B68" s="50" t="inlineStr">
         <is>
-          <t>Fore/aft (top rail) and port/starboard (forward cross arm)</t>
+          <t>Aft 13 in of the 2 x 3 inner rail on a 1/2 in 316 pin through 1/4 in lugs and a U-bracket on the aft cross arm; pad 1/2 in ply, 2 in foam, marine vinyl; detent pin for the up position</t>
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D68" s="52" t="inlineStr">
         <is>
-          <t>ea</t>
+          <t>lot</t>
         </is>
       </c>
       <c r="E68" s="53" t="n">
-        <v>25</v>
+        <v>85</v>
       </c>
       <c r="F68" s="54">
         <f>C68*E68</f>
         <v/>
       </c>
       <c r="G68" s="55" t="n">
-        <v>0.6</v>
+        <v>4.5</v>
       </c>
       <c r="H68" s="52" t="inlineStr">
         <is>
@@ -5612,19 +5644,19 @@
       <c r="I68" s="52" t="n"/>
       <c r="J68" s="50" t="inlineStr">
         <is>
-          <t>For trimming loads</t>
+          <t>Swings up and aft 95 deg so the driver can get into the seat; rests on the bracket end plate when down</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="50" t="inlineStr">
         <is>
-          <t>LED light bar 30 in, 180 W, marine</t>
+          <t>Grip (hand-hold), Hurst style</t>
         </is>
       </c>
       <c r="B69" s="50" t="inlineStr">
         <is>
-          <t>On clamp brackets above the front cage hoop</t>
+          <t>1-1/8 in 316 SS rod, bent, welded to a 3 x 2 x 1/4 in 316 base plate; 4 x 1/4 in 316 bolts through the console top and both rail walls with crush tubes, Tef-Gel and a gasket; 1-7/8 in white ball knob</t>
         </is>
       </c>
       <c r="C69" s="51" t="n">
@@ -5636,14 +5668,14 @@
         </is>
       </c>
       <c r="E69" s="53" t="n">
-        <v>170</v>
+        <v>85</v>
       </c>
       <c r="F69" s="54">
         <f>C69*E69</f>
         <v/>
       </c>
       <c r="G69" s="55" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="H69" s="52" t="inlineStr">
         <is>
@@ -5653,19 +5685,19 @@
       <c r="I69" s="52" t="n"/>
       <c r="J69" s="50" t="inlineStr">
         <is>
-          <t>About 13 A</t>
+          <t>Stainless cannot be welded to the 6061 rail; sized for 600 lbf (factor 2.2 on yield); knob position from drv_reach</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="50" t="inlineStr">
         <is>
-          <t>Searchlight 6 in LED + turret, yoke and trunnions</t>
+          <t>Transom stiffener, 6061 flat bar 3/8 x 2 in</t>
         </is>
       </c>
       <c r="B70" s="50" t="inlineStr">
         <is>
-          <t>Yaw +-180 deg, pitch +-45 deg; DIY mount</t>
+          <t>Vertical, riveted to the transom inside face behind the trim-tab bracket, bottom frame angle to rub rail (15.3 in)</t>
         </is>
       </c>
       <c r="C70" s="51" t="n">
@@ -5673,18 +5705,18 @@
       </c>
       <c r="D70" s="52" t="inlineStr">
         <is>
-          <t>lot</t>
+          <t>ea</t>
         </is>
       </c>
       <c r="E70" s="53" t="n">
-        <v>200</v>
+        <v>15</v>
       </c>
       <c r="F70" s="54">
         <f>C70*E70</f>
         <v/>
       </c>
       <c r="G70" s="55" t="n">
-        <v>9</v>
+        <v>1.1</v>
       </c>
       <c r="H70" s="52" t="inlineStr">
         <is>
@@ -5694,19 +5726,19 @@
       <c r="I70" s="52" t="n"/>
       <c r="J70" s="50" t="inlineStr">
         <is>
-          <t>About 4 A</t>
+          <t>Carries the tab adjuster pull (about 270 lb) that the bare 1/8 transom cannot</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="50" t="inlineStr">
         <is>
-          <t>Searchlight remote control</t>
+          <t>6061 rectangular tube 2 x 3 x 1/8 in</t>
         </is>
       </c>
       <c r="B71" s="50" t="inlineStr">
         <is>
-          <t>Housing, swing handle (pitch), twist grip (yaw)</t>
+          <t>Forward A-frame crossbar, 3 in deep (24.5 in); bottom on the tie-strut tabs</t>
         </is>
       </c>
       <c r="C71" s="51" t="n">
@@ -5714,18 +5746,18 @@
       </c>
       <c r="D71" s="52" t="inlineStr">
         <is>
-          <t>lot</t>
+          <t>ea</t>
         </is>
       </c>
       <c r="E71" s="53" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="F71" s="54">
         <f>C71*E71</f>
         <v/>
       </c>
       <c r="G71" s="55" t="n">
-        <v>1</v>
+        <v>2.8</v>
       </c>
       <c r="H71" s="52" t="inlineStr">
         <is>
@@ -5735,23 +5767,23 @@
       <c r="I71" s="52" t="n"/>
       <c r="J71" s="50" t="inlineStr">
         <is>
-          <t>On the aft cross arm</t>
+          <t>Replaces the 1-1/2 in crossbar: fatigue margin for the belt-pull pulses through the tie struts</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="50" t="inlineStr">
         <is>
-          <t>Push-pull (choke) cables, 20 ft</t>
+          <t>Dash panel</t>
         </is>
       </c>
       <c r="B72" s="50" t="inlineStr">
         <is>
-          <t>Yaw and pitch; zip-tied pair along the hull side and front hoop</t>
+          <t>1/8 in aluminium, 13.5 in wide, arched 8.5 in top; folds up 66 deg from the console top, faces the driver</t>
         </is>
       </c>
       <c r="C72" s="51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D72" s="52" t="inlineStr">
         <is>
@@ -5759,14 +5791,14 @@
         </is>
       </c>
       <c r="E72" s="53" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="F72" s="54">
         <f>C72*E72</f>
         <v/>
       </c>
       <c r="G72" s="55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H72" s="52" t="inlineStr">
         <is>
@@ -5776,19 +5808,19 @@
       <c r="I72" s="52" t="n"/>
       <c r="J72" s="50" t="inlineStr">
         <is>
-          <t>About 17 ft each installed</t>
+          <t>Tach centre, temp and fuel either side, everything else in the bottom row</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="50" t="inlineStr">
         <is>
-          <t>Power distribution hub</t>
+          <t>12 V socket and USB-A 5 V / 3 A charger, marine</t>
         </is>
       </c>
       <c r="B73" s="50" t="inlineStr">
         <is>
-          <t>12-way sealed blade fuse block with negative bus</t>
+          <t>With hinged rubber flaps; dash bottom row</t>
         </is>
       </c>
       <c r="C73" s="51" t="n">
@@ -5796,18 +5828,18 @@
       </c>
       <c r="D73" s="52" t="inlineStr">
         <is>
-          <t>ea</t>
+          <t>set</t>
         </is>
       </c>
       <c r="E73" s="53" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="F73" s="54">
         <f>C73*E73</f>
         <v/>
       </c>
       <c r="G73" s="55" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="H73" s="52" t="inlineStr">
         <is>
@@ -5817,19 +5849,19 @@
       <c r="I73" s="52" t="n"/>
       <c r="J73" s="50" t="inlineStr">
         <is>
-          <t>9 circuits used, 3 spare; see the wiring schematic</t>
+          <t>Both on the hub 20 A outlet circuit</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="50" t="inlineStr">
         <is>
-          <t>Main battery switch, 1/0-rated (300 A), sealed panel mount</t>
+          <t>Phone holder, swivel</t>
         </is>
       </c>
       <c r="B74" s="50" t="inlineStr">
         <is>
-          <t>Bench front between the knees, rubber gasket; studs inside the battery bay</t>
+          <t>Ball stalk at the console front-inboard corner, faces the driver; portrait or landscape (con_phone_rot)</t>
         </is>
       </c>
       <c r="C74" s="51" t="n">
@@ -5856,21 +5888,17 @@
         </is>
       </c>
       <c r="I74" s="52" t="n"/>
-      <c r="J74" s="50" t="inlineStr">
-        <is>
-          <t>Key for daily use; main switch for battery changes and emergencies</t>
-        </is>
-      </c>
+      <c r="J74" s="50" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="50" t="inlineStr">
         <is>
-          <t>Starter fusible link + MRBF fuses</t>
+          <t>Dash switches</t>
         </is>
       </c>
       <c r="B75" s="50" t="inlineStr">
         <is>
-          <t>4 AWG fusible link at battery +; 60 A MRBF (hub feed) on the switch OUT stud; 10 A MRBF (bilge) at battery +</t>
+          <t>2 sealed OFF-LO-MED-HI rotary switches (light bar, searchlight) + sealed NAV-OFF-ANCHOR rocker; DT12 connector</t>
         </is>
       </c>
       <c r="C75" s="51" t="n">
@@ -5878,18 +5906,18 @@
       </c>
       <c r="D75" s="52" t="inlineStr">
         <is>
-          <t>lot</t>
+          <t>set</t>
         </is>
       </c>
       <c r="E75" s="53" t="n">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="F75" s="54">
         <f>C75*E75</f>
         <v/>
       </c>
       <c r="G75" s="55" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="H75" s="52" t="inlineStr">
         <is>
@@ -5897,36 +5925,40 @@
         </is>
       </c>
       <c r="I75" s="52" t="n"/>
-      <c r="J75" s="50" t="n"/>
+      <c r="J75" s="50" t="inlineStr">
+        <is>
+          <t>Dash bottom row; the rotaries set the dimmers in the battery bay</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="50" t="inlineStr">
         <is>
-          <t>Battery cable 1/0 AWG tinned marine</t>
+          <t>Bubble inclinometers</t>
         </is>
       </c>
       <c r="B76" s="50" t="inlineStr">
         <is>
-          <t>Red 14 ft (battery -&gt; switch -&gt; starter), black 12 ft (battery - -&gt; engine ground); tinned lugs, boots</t>
+          <t>Fore/aft and port/starboard, both on the console top</t>
         </is>
       </c>
       <c r="C76" s="51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D76" s="52" t="inlineStr">
         <is>
-          <t>lot</t>
+          <t>ea</t>
         </is>
       </c>
       <c r="E76" s="53" t="n">
-        <v>175</v>
+        <v>25</v>
       </c>
       <c r="F76" s="54">
         <f>C76*E76</f>
         <v/>
       </c>
       <c r="G76" s="55" t="n">
-        <v>7</v>
+        <v>0.6</v>
       </c>
       <c r="H76" s="52" t="inlineStr">
         <is>
@@ -5936,19 +5968,19 @@
       <c r="I76" s="52" t="n"/>
       <c r="J76" s="50" t="inlineStr">
         <is>
-          <t>Through the conduit and the 3-hole guard grommet</t>
+          <t>For trimming loads</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="50" t="inlineStr">
         <is>
-          <t>Cable 6 AWG tinned marine</t>
+          <t>LED light bar 30 in, 180 W, marine</t>
         </is>
       </c>
       <c r="B77" s="50" t="inlineStr">
         <is>
-          <t>Red hub feed, black hub return, 4 ft total with lugs</t>
+          <t>On clamp brackets above the front cage hoop</t>
         </is>
       </c>
       <c r="C77" s="51" t="n">
@@ -5956,18 +5988,18 @@
       </c>
       <c r="D77" s="52" t="inlineStr">
         <is>
-          <t>lot</t>
+          <t>ea</t>
         </is>
       </c>
       <c r="E77" s="53" t="n">
-        <v>25</v>
+        <v>170</v>
       </c>
       <c r="F77" s="54">
         <f>C77*E77</f>
         <v/>
       </c>
       <c r="G77" s="55" t="n">
-        <v>0.5</v>
+        <v>10</v>
       </c>
       <c r="H77" s="52" t="inlineStr">
         <is>
@@ -5975,17 +6007,21 @@
         </is>
       </c>
       <c r="I77" s="52" t="n"/>
-      <c r="J77" s="50" t="n"/>
+      <c r="J77" s="50" t="inlineStr">
+        <is>
+          <t>About 13 A</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="50" t="inlineStr">
         <is>
-          <t>Duplex 12 AWG red/black tinned marine</t>
+          <t>Searchlight 6 in LED + turret, yoke and trunnions</t>
         </is>
       </c>
       <c r="B78" s="50" t="inlineStr">
         <is>
-          <t>Outlet, EFI, start, light bar, searchlight, nav lights; 100 ft</t>
+          <t>Yaw +-180 deg, pitch +-45 deg; DIY mount</t>
         </is>
       </c>
       <c r="C78" s="51" t="n">
@@ -5993,18 +6029,18 @@
       </c>
       <c r="D78" s="52" t="inlineStr">
         <is>
-          <t>roll</t>
+          <t>lot</t>
         </is>
       </c>
       <c r="E78" s="53" t="n">
-        <v>165</v>
+        <v>200</v>
       </c>
       <c r="F78" s="54">
         <f>C78*E78</f>
         <v/>
       </c>
       <c r="G78" s="55" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="H78" s="52" t="inlineStr">
         <is>
@@ -6014,38 +6050,38 @@
       <c r="I78" s="52" t="n"/>
       <c r="J78" s="50" t="inlineStr">
         <is>
-          <t>No chassis-ground returns</t>
+          <t>About 4 A</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="50" t="inlineStr">
         <is>
-          <t>Primary 18 AWG tinned marine, 12 colours</t>
+          <t>Searchlight remote control</t>
         </is>
       </c>
       <c r="B79" s="50" t="inlineStr">
         <is>
-          <t>Key, kill, gauges, sensors (tach dark gray, temp tan, fuel pink, trouble brown-white), dimmer and relay signals, bilge, pump; 25 ft spools</t>
+          <t>Housing, swing handle (pitch), twist grip (yaw)</t>
         </is>
       </c>
       <c r="C79" s="51" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="D79" s="52" t="inlineStr">
         <is>
-          <t>spool</t>
+          <t>lot</t>
         </is>
       </c>
       <c r="E79" s="53" t="n">
-        <v>12</v>
+        <v>60</v>
       </c>
       <c r="F79" s="54">
         <f>C79*E79</f>
         <v/>
       </c>
       <c r="G79" s="55" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="H79" s="52" t="inlineStr">
         <is>
@@ -6055,38 +6091,38 @@
       <c r="I79" s="52" t="n"/>
       <c r="J79" s="50" t="inlineStr">
         <is>
-          <t>ABYC E-11 colours</t>
+          <t>On the console top, forward of the cup holder</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="50" t="inlineStr">
         <is>
-          <t>Deutsch DT/DTP connector kit</t>
+          <t>Push-pull (choke) cables, 20 ft</t>
         </is>
       </c>
       <c r="B80" s="50" t="inlineStr">
         <is>
-          <t>DT12 x3, DT2 x4, DTP2 x7 with pins, seals and wedges; crimp tool</t>
+          <t>Yaw and pitch; zip-tied pair along the hull side and front hoop</t>
         </is>
       </c>
       <c r="C80" s="51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D80" s="52" t="inlineStr">
         <is>
-          <t>kit</t>
+          <t>ea</t>
         </is>
       </c>
       <c r="E80" s="53" t="n">
-        <v>240</v>
+        <v>35</v>
       </c>
       <c r="F80" s="54">
         <f>C80*E80</f>
         <v/>
       </c>
       <c r="G80" s="55" t="n">
-        <v>0.8</v>
+        <v>2</v>
       </c>
       <c r="H80" s="52" t="inlineStr">
         <is>
@@ -6096,19 +6132,19 @@
       <c r="I80" s="52" t="n"/>
       <c r="J80" s="50" t="inlineStr">
         <is>
-          <t>Every break outside the battery bay</t>
+          <t>About 17 ft each installed</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="50" t="inlineStr">
         <is>
-          <t>Looms, conduit, glands, grommets</t>
+          <t>Power distribution hub</t>
         </is>
       </c>
       <c r="B81" s="50" t="inlineStr">
         <is>
-          <t>Split loom 5/8 in and 3/8 in; 1-1/2 in sch 40 PVC conduit 3 ft with 3-hole gland caps; 2 PG13 glands; 3-hole guard grommet; aluminium deck cable cover</t>
+          <t>12-way sealed blade fuse block with negative bus</t>
         </is>
       </c>
       <c r="C81" s="51" t="n">
@@ -6116,18 +6152,18 @@
       </c>
       <c r="D81" s="52" t="inlineStr">
         <is>
-          <t>lot</t>
+          <t>ea</t>
         </is>
       </c>
       <c r="E81" s="53" t="n">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="F81" s="54">
         <f>C81*E81</f>
         <v/>
       </c>
       <c r="G81" s="55" t="n">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="H81" s="52" t="inlineStr">
         <is>
@@ -6135,17 +6171,21 @@
         </is>
       </c>
       <c r="I81" s="52" t="n"/>
-      <c r="J81" s="50" t="n"/>
+      <c r="J81" s="50" t="inlineStr">
+        <is>
+          <t>9 circuits used, 3 spare; see the wiring schematic</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="50" t="inlineStr">
         <is>
-          <t>Relays and dimmers, sealed</t>
+          <t>Main battery switch, 1/0-rated (300 A), sealed panel mount</t>
         </is>
       </c>
       <c r="B82" s="50" t="inlineStr">
         <is>
-          <t>4 x 12 V 40 A relays (start, EFI main, fuel pump, nav); 2 x IP67 20 A PWM dimmers with 3-wire remote input</t>
+          <t>Bench front between the knees, rubber gasket; studs inside the battery bay</t>
         </is>
       </c>
       <c r="C82" s="51" t="n">
@@ -6153,18 +6193,18 @@
       </c>
       <c r="D82" s="52" t="inlineStr">
         <is>
-          <t>lot</t>
+          <t>ea</t>
         </is>
       </c>
       <c r="E82" s="53" t="n">
-        <v>120</v>
+        <v>45</v>
       </c>
       <c r="F82" s="54">
         <f>C82*E82</f>
         <v/>
       </c>
       <c r="G82" s="55" t="n">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="H82" s="52" t="inlineStr">
         <is>
@@ -6174,19 +6214,19 @@
       <c r="I82" s="52" t="n"/>
       <c r="J82" s="50" t="inlineStr">
         <is>
-          <t>Inside the battery bay</t>
+          <t>Key for daily use; main switch for battery changes and emergencies</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="50" t="inlineStr">
         <is>
-          <t>Bilge float switch + AUTO-OFF-MAN switch</t>
+          <t>Starter fusible link + MRBF fuses</t>
         </is>
       </c>
       <c r="B83" s="50" t="inlineStr">
         <is>
-          <t>Float in the sump; sealed toggle on the bench front</t>
+          <t>4 AWG fusible link at battery +; 60 A MRBF (hub feed) on the switch OUT stud; 10 A MRBF (bilge) at battery +</t>
         </is>
       </c>
       <c r="C83" s="51" t="n">
@@ -6194,18 +6234,18 @@
       </c>
       <c r="D83" s="52" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>lot</t>
         </is>
       </c>
       <c r="E83" s="53" t="n">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="F83" s="54">
         <f>C83*E83</f>
         <v/>
       </c>
       <c r="G83" s="55" t="n">
-        <v>0.7</v>
+        <v>0.4</v>
       </c>
       <c r="H83" s="52" t="inlineStr">
         <is>
@@ -6213,21 +6253,17 @@
         </is>
       </c>
       <c r="I83" s="52" t="n"/>
-      <c r="J83" s="50" t="inlineStr">
-        <is>
-          <t>Always on through its own 10 A fuse</t>
-        </is>
-      </c>
+      <c r="J83" s="50" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="50" t="inlineStr">
         <is>
-          <t>Fuel pump and filter, EFI inline</t>
+          <t>Battery cable 1/0 AWG tinned marine</t>
         </is>
       </c>
       <c r="B84" s="50" t="inlineStr">
         <is>
-          <t>On a bracket on the port engine-bed plate, outside the guard</t>
+          <t>Red 14 ft (battery -&gt; switch -&gt; starter), black 12 ft (battery - -&gt; engine ground); tinned lugs, boots</t>
         </is>
       </c>
       <c r="C84" s="51" t="n">
@@ -6235,18 +6271,18 @@
       </c>
       <c r="D84" s="52" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>lot</t>
         </is>
       </c>
       <c r="E84" s="53" t="n">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="F84" s="54">
         <f>C84*E84</f>
         <v/>
       </c>
       <c r="G84" s="55" t="n">
-        <v>2.5</v>
+        <v>7</v>
       </c>
       <c r="H84" s="52" t="inlineStr">
         <is>
@@ -6256,19 +6292,19 @@
       <c r="I84" s="52" t="n"/>
       <c r="J84" s="50" t="inlineStr">
         <is>
-          <t>Delete if the drivetrain list already carries them</t>
+          <t>Through the conduit and the 3-hole guard grommet</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="50" t="inlineStr">
         <is>
-          <t>Fuel sender, electric 240-33 ohm</t>
+          <t>Cable 6 AWG tinned marine</t>
         </is>
       </c>
       <c r="B85" s="50" t="inlineStr">
         <is>
-          <t>In the portable tank, DT2 at the tank front</t>
+          <t>Red hub feed, black hub return, 4 ft total with lugs</t>
         </is>
       </c>
       <c r="C85" s="51" t="n">
@@ -6276,18 +6312,18 @@
       </c>
       <c r="D85" s="52" t="inlineStr">
         <is>
-          <t>ea</t>
+          <t>lot</t>
         </is>
       </c>
       <c r="E85" s="53" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="F85" s="54">
         <f>C85*E85</f>
         <v/>
       </c>
       <c r="G85" s="55" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="H85" s="52" t="inlineStr">
         <is>
@@ -6295,21 +6331,17 @@
         </is>
       </c>
       <c r="I85" s="52" t="n"/>
-      <c r="J85" s="50" t="inlineStr">
-        <is>
-          <t>The tank must accept a sender</t>
-        </is>
-      </c>
+      <c r="J85" s="50" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="50" t="inlineStr">
         <is>
-          <t>Nav lights</t>
+          <t>Duplex 12 AWG red/black tinned marine</t>
         </is>
       </c>
       <c r="B86" s="50" t="inlineStr">
         <is>
-          <t>Bow red/green combination on a 12 in stanchion; all-round white on an 18 in mast with U-bolt saddle on the aft hoop</t>
+          <t>Outlet, EFI, start, light bar, searchlight, nav lights; 100 ft</t>
         </is>
       </c>
       <c r="C86" s="51" t="n">
@@ -6317,18 +6349,18 @@
       </c>
       <c r="D86" s="52" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>roll</t>
         </is>
       </c>
       <c r="E86" s="53" t="n">
-        <v>140</v>
+        <v>165</v>
       </c>
       <c r="F86" s="54">
         <f>C86*E86</f>
         <v/>
       </c>
       <c r="G86" s="55" t="n">
-        <v>2.5</v>
+        <v>6</v>
       </c>
       <c r="H86" s="52" t="inlineStr">
         <is>
@@ -6338,38 +6370,38 @@
       <c r="I86" s="52" t="n"/>
       <c r="J86" s="50" t="inlineStr">
         <is>
-          <t>USCG Rule 23 for power vessels under 12 m</t>
+          <t>No chassis-ground returns</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="50" t="inlineStr">
         <is>
-          <t>Marine plywood 1/2 in, 4x8</t>
+          <t>Primary 18 AWG tinned marine, 12 colours</t>
         </is>
       </c>
       <c r="B87" s="50" t="inlineStr">
         <is>
-          <t>Bench bottom panel, bay bulkhead, both lids</t>
+          <t>Key, kill, gauges, sensors (tach dark gray, temp tan, fuel pink, trouble brown-white), dimmer and relay signals, bilge, pump; 25 ft spools</t>
         </is>
       </c>
       <c r="C87" s="51" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D87" s="52" t="inlineStr">
         <is>
-          <t>sheet</t>
+          <t>spool</t>
         </is>
       </c>
       <c r="E87" s="53" t="n">
-        <v>150</v>
+        <v>12</v>
       </c>
       <c r="F87" s="54">
         <f>C87*E87</f>
         <v/>
       </c>
       <c r="G87" s="55" t="n">
-        <v>7.5</v>
+        <v>0.4</v>
       </c>
       <c r="H87" s="52" t="inlineStr">
         <is>
@@ -6379,19 +6411,19 @@
       <c r="I87" s="52" t="n"/>
       <c r="J87" s="50" t="inlineStr">
         <is>
-          <t>Epoxy-coat inside the cooler</t>
+          <t>ABYC E-11 colours</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="50" t="inlineStr">
         <is>
-          <t>Deck hardware</t>
+          <t>Deutsch DT/DTP connector kit</t>
         </is>
       </c>
       <c r="B88" s="50" t="inlineStr">
         <is>
-          <t>4 in aluminium cleats (4), 1/4 in bow knees (2), 316 bow-eye strap and 2 in ring</t>
+          <t>DT12 x3, DT2 x4, DTP2 x7 with pins, seals and wedges; crimp tool</t>
         </is>
       </c>
       <c r="C88" s="51" t="n">
@@ -6399,18 +6431,18 @@
       </c>
       <c r="D88" s="52" t="inlineStr">
         <is>
-          <t>lot</t>
+          <t>kit</t>
         </is>
       </c>
       <c r="E88" s="53" t="n">
-        <v>110</v>
+        <v>240</v>
       </c>
       <c r="F88" s="54">
         <f>C88*E88</f>
         <v/>
       </c>
       <c r="G88" s="55" t="n">
-        <v>4</v>
+        <v>0.8</v>
       </c>
       <c r="H88" s="52" t="inlineStr">
         <is>
@@ -6420,19 +6452,19 @@
       <c r="I88" s="52" t="n"/>
       <c r="J88" s="50" t="inlineStr">
         <is>
-          <t>Bow cleats on the knees, stern cleats on the transom corners</t>
+          <t>Every break outside the battery bay</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="50" t="inlineStr">
         <is>
-          <t>Fire extinguisher, USCG B-1 (5-B:C) marine</t>
+          <t>Looms, conduit, glands, grommets</t>
         </is>
       </c>
       <c r="B89" s="50" t="inlineStr">
         <is>
-          <t>With quick-release bracket</t>
+          <t>Split loom 5/8 in and 3/8 in; 1-1/2 in sch 40 PVC conduit 3 ft with 3-hole gland caps; 2 PG13 glands; 3-hole guard grommet; aluminium deck cable cover</t>
         </is>
       </c>
       <c r="C89" s="51" t="n">
@@ -6440,18 +6472,18 @@
       </c>
       <c r="D89" s="52" t="inlineStr">
         <is>
-          <t>ea</t>
+          <t>lot</t>
         </is>
       </c>
       <c r="E89" s="53" t="n">
-        <v>40</v>
+        <v>95</v>
       </c>
       <c r="F89" s="54">
         <f>C89*E89</f>
         <v/>
       </c>
       <c r="G89" s="55" t="n">
-        <v>4.5</v>
+        <v>2.5</v>
       </c>
       <c r="H89" s="52" t="inlineStr">
         <is>
@@ -6459,21 +6491,17 @@
         </is>
       </c>
       <c r="I89" s="52" t="n"/>
-      <c r="J89" s="50" t="inlineStr">
-        <is>
-          <t>Bow shelf, starboard of the tank</t>
-        </is>
-      </c>
+      <c r="J89" s="50" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="50" t="inlineStr">
         <is>
-          <t>Air horn, 8 oz can</t>
+          <t>Relays and dimmers, sealed</t>
         </is>
       </c>
       <c r="B90" s="50" t="inlineStr">
         <is>
-          <t>With bracket</t>
+          <t>5 x 12 V 40 A relays (start, EFI main, fuel pump, nav, anchor) + 2 x 1N5408 diodes; 2 x IP67 20 A PWM dimmers with 3-wire remote input</t>
         </is>
       </c>
       <c r="C90" s="51" t="n">
@@ -6481,18 +6509,18 @@
       </c>
       <c r="D90" s="52" t="inlineStr">
         <is>
-          <t>ea</t>
+          <t>lot</t>
         </is>
       </c>
       <c r="E90" s="53" t="n">
-        <v>25</v>
+        <v>140</v>
       </c>
       <c r="F90" s="54">
         <f>C90*E90</f>
         <v/>
       </c>
       <c r="G90" s="55" t="n">
-        <v>0.8</v>
+        <v>1.4</v>
       </c>
       <c r="H90" s="52" t="inlineStr">
         <is>
@@ -6502,19 +6530,19 @@
       <c r="I90" s="52" t="n"/>
       <c r="J90" s="50" t="inlineStr">
         <is>
-          <t>Bow shelf, port of the tank</t>
+          <t>Inside the battery bay</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="50" t="inlineStr">
         <is>
-          <t>Rev 7 fasteners</t>
+          <t>Bilge float switch + AUTO-OFF-MAN switch</t>
         </is>
       </c>
       <c r="B91" s="50" t="inlineStr">
         <is>
-          <t>SS bolts, rivnuts, U-bolts and clamps for the items above</t>
+          <t>Float in the sump; sealed toggle on the bench front</t>
         </is>
       </c>
       <c r="C91" s="51" t="n">
@@ -6522,7 +6550,7 @@
       </c>
       <c r="D91" s="52" t="inlineStr">
         <is>
-          <t>lot</t>
+          <t>set</t>
         </is>
       </c>
       <c r="E91" s="53" t="n">
@@ -6533,71 +6561,440 @@
         <v/>
       </c>
       <c r="G91" s="55" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H91" s="52" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I91" s="52" t="n"/>
+      <c r="J91" s="50" t="inlineStr">
+        <is>
+          <t>Always on through its own 10 A fuse</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="50" t="inlineStr">
+        <is>
+          <t>Fuel pump and filter, EFI inline</t>
+        </is>
+      </c>
+      <c r="B92" s="50" t="inlineStr">
+        <is>
+          <t>On a bracket on the port engine-bed plate, outside the guard</t>
+        </is>
+      </c>
+      <c r="C92" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D92" s="52" t="inlineStr">
+        <is>
+          <t>set</t>
+        </is>
+      </c>
+      <c r="E92" s="53" t="n">
+        <v>170</v>
+      </c>
+      <c r="F92" s="54">
+        <f>C92*E92</f>
+        <v/>
+      </c>
+      <c r="G92" s="55" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H92" s="52" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I92" s="52" t="n"/>
+      <c r="J92" s="50" t="inlineStr">
+        <is>
+          <t>Delete if the drivetrain list already carries them</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="50" t="inlineStr">
+        <is>
+          <t>Fuel sender, electric 240-33 ohm</t>
+        </is>
+      </c>
+      <c r="B93" s="50" t="inlineStr">
+        <is>
+          <t>In the portable tank, DT2 at the tank front</t>
+        </is>
+      </c>
+      <c r="C93" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D93" s="52" t="inlineStr">
+        <is>
+          <t>ea</t>
+        </is>
+      </c>
+      <c r="E93" s="53" t="n">
+        <v>60</v>
+      </c>
+      <c r="F93" s="54">
+        <f>C93*E93</f>
+        <v/>
+      </c>
+      <c r="G93" s="55" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H93" s="52" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I93" s="52" t="n"/>
+      <c r="J93" s="50" t="inlineStr">
+        <is>
+          <t>The tank must accept a sender</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="50" t="inlineStr">
+        <is>
+          <t>Nav lights</t>
+        </is>
+      </c>
+      <c r="B94" s="50" t="inlineStr">
+        <is>
+          <t>Bow red/green combination on a 12 in stanchion; all-round white on an 18 in mast with U-bolt saddle on the aft hoop</t>
+        </is>
+      </c>
+      <c r="C94" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D94" s="52" t="inlineStr">
+        <is>
+          <t>set</t>
+        </is>
+      </c>
+      <c r="E94" s="53" t="n">
+        <v>140</v>
+      </c>
+      <c r="F94" s="54">
+        <f>C94*E94</f>
+        <v/>
+      </c>
+      <c r="G94" s="55" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H94" s="52" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I94" s="52" t="n"/>
+      <c r="J94" s="50" t="inlineStr">
+        <is>
+          <t>USCG Rule 23 for power vessels under 12 m</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="50" t="inlineStr">
+        <is>
+          <t>Marine plywood 1/2 in, 4x8</t>
+        </is>
+      </c>
+      <c r="B95" s="50" t="inlineStr">
+        <is>
+          <t>Bench bottom panel, bay bulkhead, both lids</t>
+        </is>
+      </c>
+      <c r="C95" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D95" s="52" t="inlineStr">
+        <is>
+          <t>sheet</t>
+        </is>
+      </c>
+      <c r="E95" s="53" t="n">
+        <v>150</v>
+      </c>
+      <c r="F95" s="54">
+        <f>C95*E95</f>
+        <v/>
+      </c>
+      <c r="G95" s="55" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="H95" s="52" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I95" s="52" t="n"/>
+      <c r="J95" s="50" t="inlineStr">
+        <is>
+          <t>Epoxy-coat inside the cooler</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="50" t="inlineStr">
+        <is>
+          <t>Deck hardware</t>
+        </is>
+      </c>
+      <c r="B96" s="50" t="inlineStr">
+        <is>
+          <t>4 in aluminium cleats (4), 1/4 in bow knees (2), 316 bow-eye strap and 2 in ring</t>
+        </is>
+      </c>
+      <c r="C96" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D96" s="52" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="E96" s="53" t="n">
+        <v>110</v>
+      </c>
+      <c r="F96" s="54">
+        <f>C96*E96</f>
+        <v/>
+      </c>
+      <c r="G96" s="55" t="n">
+        <v>4</v>
+      </c>
+      <c r="H96" s="52" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I96" s="52" t="n"/>
+      <c r="J96" s="50" t="inlineStr">
+        <is>
+          <t>Bow cleats on the knees, stern cleats on the transom corners</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="50" t="inlineStr">
+        <is>
+          <t>Fire extinguisher, USCG B-1 (5-B:C) marine</t>
+        </is>
+      </c>
+      <c r="B97" s="50" t="inlineStr">
+        <is>
+          <t>With quick-release bracket</t>
+        </is>
+      </c>
+      <c r="C97" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D97" s="52" t="inlineStr">
+        <is>
+          <t>ea</t>
+        </is>
+      </c>
+      <c r="E97" s="53" t="n">
+        <v>40</v>
+      </c>
+      <c r="F97" s="54">
+        <f>C97*E97</f>
+        <v/>
+      </c>
+      <c r="G97" s="55" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H97" s="52" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I97" s="52" t="n"/>
+      <c r="J97" s="50" t="inlineStr">
+        <is>
+          <t>Bow shelf, starboard of the tank</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="50" t="inlineStr">
+        <is>
+          <t>Air horn, 8 oz can</t>
+        </is>
+      </c>
+      <c r="B98" s="50" t="inlineStr">
+        <is>
+          <t>With bracket</t>
+        </is>
+      </c>
+      <c r="C98" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D98" s="52" t="inlineStr">
+        <is>
+          <t>ea</t>
+        </is>
+      </c>
+      <c r="E98" s="53" t="n">
+        <v>25</v>
+      </c>
+      <c r="F98" s="54">
+        <f>C98*E98</f>
+        <v/>
+      </c>
+      <c r="G98" s="55" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H98" s="52" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I98" s="52" t="n"/>
+      <c r="J98" s="50" t="inlineStr">
+        <is>
+          <t>Bow shelf, port of the tank</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="50" t="inlineStr">
+        <is>
+          <t>Flag staff and international-orange flag</t>
+        </is>
+      </c>
+      <c r="B99" s="50" t="inlineStr">
+        <is>
+          <t>3/4 in 6061 tube removable staff in a 7/8 in socket on a U-bolt saddle on the aft hoop, 12 in port of the stern light; 12 x 10 in nylon flag, bottom edge 122 in above the hull bottom</t>
+        </is>
+      </c>
+      <c r="C99" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D99" s="52" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="E99" s="53" t="n">
+        <v>45</v>
+      </c>
+      <c r="F99" s="54">
+        <f>C99*E99</f>
+        <v/>
+      </c>
+      <c r="G99" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="H99" s="52" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I99" s="52" t="n"/>
+      <c r="J99" s="50" t="inlineStr">
+        <is>
+          <t>Florida Statute 327.391: flag at least 10 x 12 in, at least 10 ft above the lowest part of the boat; pull the staff to trailer</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="50" t="inlineStr">
+        <is>
+          <t>Rev 7 fasteners</t>
+        </is>
+      </c>
+      <c r="B100" s="50" t="inlineStr">
+        <is>
+          <t>SS bolts, rivnuts, U-bolts and clamps for the items above</t>
+        </is>
+      </c>
+      <c r="C100" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D100" s="52" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="E100" s="53" t="n">
+        <v>60</v>
+      </c>
+      <c r="F100" s="54">
+        <f>C100*E100</f>
+        <v/>
+      </c>
+      <c r="G100" s="55" t="n">
         <v>2</v>
       </c>
-      <c r="H91" s="52" t="inlineStr">
+      <c r="H100" s="52" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="I91" s="52" t="n"/>
-      <c r="J91" s="50" t="n"/>
-    </row>
-    <row r="92"/>
-    <row r="93">
-      <c r="A93" s="38" t="inlineStr">
+      <c r="I100" s="52" t="n"/>
+      <c r="J100" s="50" t="n"/>
+    </row>
+    <row r="101"/>
+    <row r="102">
+      <c r="A102" s="38" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B93" s="38" t="n"/>
-      <c r="C93" s="38" t="n"/>
-      <c r="D93" s="38" t="n"/>
-      <c r="E93" s="38" t="n"/>
-      <c r="F93" s="39">
-        <f>SUM(F5:F91)</f>
-        <v/>
-      </c>
-      <c r="G93" s="40">
-        <f>SUM(G5:G91)</f>
-        <v/>
-      </c>
-      <c r="H93" s="38" t="n"/>
-      <c r="I93" s="38" t="n"/>
-      <c r="J93" s="38" t="n"/>
-    </row>
-    <row r="94">
-      <c r="A94" s="35" t="inlineStr">
+      <c r="B102" s="38" t="n"/>
+      <c r="C102" s="38" t="n"/>
+      <c r="D102" s="38" t="n"/>
+      <c r="E102" s="38" t="n"/>
+      <c r="F102" s="39">
+        <f>SUM(F5:F100)</f>
+        <v/>
+      </c>
+      <c r="G102" s="40">
+        <f>SUM(G5:G100)</f>
+        <v/>
+      </c>
+      <c r="H102" s="38" t="n"/>
+      <c r="I102" s="38" t="n"/>
+      <c r="J102" s="38" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="35" t="inlineStr">
         <is>
           <t>Weight included in the CAD model</t>
         </is>
       </c>
-      <c r="G94" s="59">
-        <f>SUMIF(H5:H91,"Y",G5:G91)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="35" t="inlineStr">
+      <c r="G103" s="59">
+        <f>SUMIF(H5:H100,"Y",G5:G100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="35" t="inlineStr">
         <is>
           <t>Weight not in the CAD model (fasteners, paint, wiring)</t>
         </is>
       </c>
-      <c r="G95" s="59">
-        <f>SUMIF(H5:H91,"N",G5:G91)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="35" t="inlineStr">
+      <c r="G104" s="59">
+        <f>SUMIF(H5:H100,"N",G5:G100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="35" t="inlineStr">
         <is>
           <t>CAD model weight for this group (reference)</t>
         </is>
       </c>
-      <c r="G96" s="46" t="n">
+      <c r="G105" s="46" t="n">
         <v>322.87</v>
       </c>
-      <c r="J96" s="33" t="inlineStr">
+      <c r="J105" s="33" t="inlineStr">
         <is>
           <t>Rev 6 CAD weight reports; rev 7 lines above are model volumes or catalog weights</t>
         </is>

</xml_diff>